<commit_message>
v3: simulador em paisagem com aba Fábrica, portal (tema, cor, informações na tela, restaurar fábrica), E2E/crosscheck, docs de hardware/bancada/fábrica e lista de materiais ES3C28P
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01N4nRHLvd7LEdWA14RQqaQ3
</commit_message>
<xml_diff>
--- a/docs/lista_de_materiais.xlsx
+++ b/docs/lista_de_materiais.xlsx
@@ -22,12 +22,12 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="147" uniqueCount="121">
-  <si>
-    <t xml:space="preserve">TubaBot v2 — lista de materiais (Brasil)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preços em R$ são FAIXAS ESTIMADAS (out/2026) a partir de preços oficiais e de lojas pesquisadas. As páginas do Mercado Livre e da Shopee não puderam ser abertas deste ambiente, então os links levam a buscas já filtradas: 'menor preço' e 'mais vendidos/relevantes' (que puxam os anúncios com mais avaliações). Confira no anúncio: avaliação ≥ 4,5, mais de 50 vendas, e a especificação da coluna 'Conferir no anúncio'.</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="141" uniqueCount="113">
+  <si>
+    <t xml:space="preserve">TubaBot v3 (ES3C28P) — lista de materiais por unidade (Brasil)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Preços em R$ são FAIXAS ESTIMADAS (out/2026) a partir de preços internacionais pesquisados. As páginas do Mercado Livre e da Shopee não puderam ser abertas deste ambiente: os links levam a buscas já filtradas por 'menor preço' e por 'mais vendidos/relevantes' (os anúncios com mais avaliações). Confira no anúncio: nota ≥ 4,5, mais de 50 vendas e a especificação da coluna 'Conferir no anúncio'. Lite = sem bateria; Pro = com bateria.</t>
   </si>
   <si>
     <t xml:space="preserve">#</t>
@@ -39,7 +39,7 @@
     <t xml:space="preserve">Qtd</t>
   </si>
   <si>
-    <t xml:space="preserve">Obrigatório?</t>
+    <t xml:space="preserve">Lite / Pro</t>
   </si>
   <si>
     <t xml:space="preserve">Especificação exata</t>
@@ -69,16 +69,16 @@
     <t xml:space="preserve">Observações</t>
   </si>
   <si>
-    <t xml:space="preserve">Placa Waveshare ESP32-S3-Touch-AMOLED-1.75 (SKU 31261)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sim</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ESP32-S3R8, 8 MB PSRAM, 16 MB flash, AMOLED 1,75" 466×466 CO5300, toque CST9217, IMU QMI8658, AXP2101, RTC PCF85063, ES8311 + ES7210 (2 microfones), USB-C</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Nome exato 'ESP32-S3-Touch-AMOLED-1.75' (NÃO 1.43, NÃO 1.75C). Versão padrão 31261, sem case. GPS (31264) também serve, mas é mais cara.</t>
+    <t xml:space="preserve">Placa ES3C28P — ESP32-S3 + tela IPS 2,8" 240×320 com TOQUE CAPACITIVO</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lite e Pro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESP32-S3R8 (16 MB flash, 8 MB PSRAM), ILI9341V, toque FT6336G, codec ES8311 + amplificador + microfone, conector de alto-falante, conector de bateria com carregador TP4054, USB-C</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Modelo exato ES3C28P (o 'C' = capacitivo). NÃO comprar ES3N28P (sem toque) nem a 'ESP32-S3-Touch-LCD-2.8' da Waveshare (outra placa). A foto deve mostrar os conectores SPEAKER e BAT.</t>
   </si>
   <si>
     <t xml:space="preserve">ML · menor preço</t>
@@ -90,151 +90,124 @@
     <t xml:space="preserve">Shopee · mais vendidos</t>
   </si>
   <si>
-    <t xml:space="preserve">Waveshare oficial (US$ 29,99 + frete)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Item principal. Se não houver no ML/Shopee com bom vendedor, a loja oficial da Waveshare ou AliExpress (loja oficial Waveshare) costuma sair mais barato com o Remessa Conforme.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bateria LiPo 3,7 V 803040 1000 mAh com plugue MX1.25</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sim (para usar sem cabo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">LiPo 3,7 V, 1000 mAh, tamanho 8 × 30 × 40 mm (803040), circuito de proteção (PCM), 2 fios</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Tamanho máx. ~8×30×40 mm para caber no corpo Neo; COM proteção; plugue MX1.25 (1,25 mm). Ao receber, confira a polaridade com o multímetro antes de plugar.</t>
+    <t xml:space="preserve">AliExpress — busca ES3C28P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Referência internacional ~US$ 15 (fabricante QDtech/LCDWIKI). No AliExpress com o Remessa Conforme costuma sair mais barato que no ML.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alto-falante 8 Ω 1,5–2 W (ou 4 Ω 2 W), pequeno</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cápsula 28–40 mm ou retangular 20×30 mm; 8 Ω 1,5 W ou 4 Ω 2 W (valores da LCDWIKI)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Impedância e potência; já com fios. Confira o plugue do conector SPEAKER da sua placa (MX1.25 ou PH2.0) — se não bater, use o kit de rabichos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Busca geral ML (alto-falante 8 Ω 2 W)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kits com 2–5 unidades costumam custar o mesmo que uma.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bateria LiPo 3,7 V 1000–1500 mAh</t>
+  </si>
+  <si>
+    <t xml:space="preserve">só Pro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LiPo 1S 3,7 V com proteção (PCM); 1000 a 1500 mAh; espessura conforme o corpo (ex.: 103040, 803450)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">COM proteção; tamanho que caiba no corpo; plugue compatível com o conector BAT (MX1.25 ou PH2.0). Antes de plugar, confira a polaridade com o multímetro.</t>
   </si>
   <si>
     <t xml:space="preserve">Busca geral ML (bateria 3,7 V 1000 mAh)</t>
   </si>
   <si>
-    <t xml:space="preserve">Se vier com plugue PH2.0/JST, use o kit de rabichos MX1.25 (item 4). Nunca inverta + e −.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Alto-falante 8 Ω 2 W (28 mm redondo ou cápsula 2030)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sim (para ter som)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8 Ω, 1 a 2 W, diâmetro 28 mm (ou retangular 20×30 mm), fino</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Impedância 8 Ω; potência 1–2 W; tamanho pequeno. Melhor se já vier com fios/plugue MX1.25.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Busca geral ML (alto-falante 8 Ω 2 W)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kits com 2–5 unidades costumam custar o mesmo que uma.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kit de rabichos (pigtails) MX1.25 2 pinos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Recomendado</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conector Molex PicoBlade / MX1.25 mm, 2 vias, fêmea com fio 10–15 cm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Passo 1,25 mm (não confundir com PH2.0 nem JST-SH 1,0 mm). Kit com 10 pares.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Para adaptar bateria e alto-falante se vierem com outro plugue. Exige solda simples (ferro da v1).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Arquivos 3D do corpo Neo Deskimon (STL)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sim (corpo)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Modelo Neo da Creative Chance (capuz com fones), feito para a placa Waveshare 1.75</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Comprar direto da Creative Chance (Thangs).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Creative Chance — Neo Deskimon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Preço de referência ~US$ 7,99 (Thangs). Uso pessoal; não revender o STL.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Impressão 3D do corpo (serviço) — OU filamento PLA 1 kg</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sim (uma das duas)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PLA, 0,2 mm, 15–20 % preenchimento; cor à escolha</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Serviço: envie o STL, peça PLA e prazo. Filamento: PLA 1,75 mm de marca com boas avaliações.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Filamento PLA 1,75 mm — busca ML</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Só compre filamento se tiver impressora (ou amigo com impressora). Bambu PLA Lite 1 kg foi visto por ~R$ 110.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fita dupla-face fina (espuma 0,8–1 mm)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fita dupla-face de espuma fina, 12 mm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Espessura ≤ 1 mm para não empurrar a placa.</t>
+    <t xml:space="preserve">O carregador da placa (TP4054) carrega a até ~0,5 A: 1000–1500 mAh carregam em 2–4 h.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kit de rabichos MX1.25 e PH2.0 de 2 vias</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conectores 2 vias com fio (passo 1,25 mm e 2,0 mm)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Um kit com os dois passos resolve qualquer diferença entre placa, alto-falante e bateria.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Exige solda simples (o ferro da v1 serve). Serve para muitas unidades.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filamento PLA 1,75 mm na cor do corpo (ou impressão sob encomenda)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLA 1 kg nas cores do produto: vermelho, azul, branco ou grafite/preto</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PLA de marca com boas avaliações, na cor da variante. Serviço: envie o STL do corpo do TubaBot.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Filamento PLA — busca ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Um corpo usa ~40–80 g: 1 kg rende vários TubaBots (mínimo = custo por unidade).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Parafusos M2 × 6 mm (ou M2,5) + porcas/insertos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Para os 4 furos da placa ES3C28P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Confira o diâmetro dos furos da sua placa (M2 ou M2,5).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kits sortidos M2/M2,5 servem para muitas unidades (preço por parafuso).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fita dupla-face de espuma fina</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fita dupla-face de espuma, 0,8–1 mm, 12 mm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Espessura ≤ 1 mm.</t>
   </si>
   <si>
     <t xml:space="preserve">Prende a bateria no corpo, longe de cantos vivos.</t>
   </si>
   <si>
-    <t xml:space="preserve">TOTAL estimado (itens novos)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Peças da v1 que você já tem (não comprar)</t>
+    <t xml:space="preserve">TOTAL estimado — TubaBot Lite</t>
+  </si>
+  <si>
+    <t xml:space="preserve">TOTAL estimado — TubaBot Pro</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Peças da v1 (não comprar)</t>
   </si>
   <si>
     <t xml:space="preserve">Situação</t>
   </si>
   <si>
-    <t xml:space="preserve">Uso na v2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Motor de vibração MV50</t>
+    <t xml:space="preserve">Uso na v3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cabo USB-C de dados (Ugreen US287)</t>
   </si>
   <si>
     <t xml:space="preserve">JÁ TENHO (v1)</t>
   </si>
   <si>
-    <t xml:space="preserve">Opcional — firmware 'tubabot_vibra', ligar IN→GPIO16, VCC→3V3, GND→GND.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jumpers fêmea-fêmea 10 cm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Para o MV50.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cabo USB-C de dados (Ugreen US287)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Gravação, alimentação, carga.</t>
+    <t xml:space="preserve">Gravação, alimentação e carga (Pro).</t>
   </si>
   <si>
     <t xml:space="preserve">Multímetro Kapbom DT-9205A</t>
   </si>
   <si>
-    <t xml:space="preserve">Conferir polaridade da bateria.</t>
+    <t xml:space="preserve">Conferir a polaridade da bateria.</t>
   </si>
   <si>
     <t xml:space="preserve">Ferro de solda 60 W + estanho</t>
@@ -246,7 +219,16 @@
     <t xml:space="preserve">Ímãs de neodímio 8×2 mm</t>
   </si>
   <si>
-    <t xml:space="preserve">Opcional: fecho da tampa traseira.</t>
+    <t xml:space="preserve">Opcional: fecho do corpo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ESP32-C3, OLED 0,96", TTP223, buzzer, motor MV50</t>
+  </si>
+  <si>
+    <t xml:space="preserve">NÃO USADOS na v3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Toda a interação agora é pela tela de toque.</t>
   </si>
   <si>
     <t xml:space="preserve">Critério</t>
@@ -267,22 +249,22 @@
     <t xml:space="preserve">Confirma que chega o item da foto</t>
   </si>
   <si>
-    <t xml:space="preserve">Foto mostra o nome 'ESP32-S3-Touch-AMOLED-1.75' na placa/caixa</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Existem as versões 1.43 e 1.75C, que não servem no corpo</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bateria: tamanho 803040 e 'com proteção'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cabe no corpo e é segura</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Conector MX1.25 (1,25 mm) — se não informar, pergunte</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PH2.0 e JST-SH não encaixam na placa</t>
+    <t xml:space="preserve">Placa: o nome ES3C28P aparece no anúncio/placa (C = toque capacitivo)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ES3N28P não tem toque; a Waveshare 2.8 é outra placa, com outros pinos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bateria (Pro): 'com proteção' e tamanho que caiba no corpo</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Segurança e encaixe</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conectores SPEAKER e BAT: pergunte ao vendedor se são MX1.25 ou PH2.0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Os dois são comuns nesta família de placas</t>
   </si>
   <si>
     <t xml:space="preserve">Prefira 'Full' (ML) ou envio nacional</t>
@@ -297,10 +279,10 @@
     <t xml:space="preserve">Imposto já incluso no preço exibido</t>
   </si>
   <si>
-    <t xml:space="preserve">Compare preço + frete; kits de 2–5 alto-falantes/rabichos costumam compensar</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Sobra peça de reposição</t>
+    <t xml:space="preserve">Compare preço + frete; kits de alto-falantes/rabichos/parafusos compensam</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Sobra peça para as próximas unidades</t>
   </si>
   <si>
     <t xml:space="preserve">Fonte</t>
@@ -312,55 +294,49 @@
     <t xml:space="preserve">O que foi usado</t>
   </si>
   <si>
-    <t xml:space="preserve">Waveshare — página do produto</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.waveshare.com/esp32-s3-touch-amoled-1.75.htm</t>
-  </si>
-  <si>
-    <t xml:space="preserve">preço oficial (US$ 29,99 a 39,99), SKUs 31261/31262/31264</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waveshare — documentação</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://docs.waveshare.com/ESP32-S3-Touch-AMOLED-1.75</t>
-  </si>
-  <si>
-    <t xml:space="preserve">especificações, conectores</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Waveshare — repositório oficial</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://github.com/waveshareteam/ESP32-S3-Touch-AMOLED-1.75</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pinos e bibliotecas usados no firmware</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://creative-chance.com/en-brl/products/neo-deskimon</t>
-  </si>
-  <si>
-    <t xml:space="preserve">corpo de referência</t>
-  </si>
-  <si>
-    <t xml:space="preserve">eBay (referência de preço internacional)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.ebay.com/itm/267546467085</t>
-  </si>
-  <si>
-    <t xml:space="preserve">US$ 47,84 + frete (versão 1.75C)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Amazon US (referência)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://www.amazon.com/AmpOhm360-Waveshare-Development-Microphones-Interface/dp/B0H97CDMKS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">versão com case (31262), indisponível na consulta</t>
+    <t xml:space="preserve">LCDWIKI — 2.8inch ESP32-S3 Display (ES3C28P)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.lcdwiki.com/2.8inch_ESP32-S3_Display</t>
+  </si>
+  <si>
+    <t xml:space="preserve">especificações e pinos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BSP ngttai/esp32_s3_es3c28p</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/ngttai/esp32_s3_es3c28p</t>
+  </si>
+  <si>
+    <t xml:space="preserve">mapa de pinos, alto-falante 8 Ω 1,5 W / 4 Ω 2 W, bateria com TP4054</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Launcher — perfil ES3C28P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/bmorcelli/Launcher/issues/373</t>
+  </si>
+  <si>
+    <t xml:space="preserve">pinos de áudio (I²S) e habilitação do amplificador</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bruce firmware — PR ES3C28P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://github.com/BruceDevices/firmware/pull/2178</t>
+  </si>
+  <si>
+    <t xml:space="preserve">preço de referência ~US$ 15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Alibaba — ES3C28P/ES3N28P</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.alibaba.com/product-detail/ES3C28P-ES3N28P-2-8-inch-ESP32_1601603512242.html</t>
+  </si>
+  <si>
+    <t xml:space="preserve">US$ 12–15 (atacado)</t>
   </si>
   <si>
     <t xml:space="preserve">Mercado Livre — bateria 3,7 V 1000 mAh</t>
@@ -864,9 +840,9 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="4"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="34"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="6"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="46"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="7" style="0" width="18"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="9" min="9" style="0" width="20"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="10" min="10" style="0" width="30"/>
@@ -894,6 +870,7 @@
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
       <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
     </row>
     <row r="4" customFormat="false" ht="33.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
@@ -936,7 +913,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="5" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="5" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="n">
         <v>1</v>
       </c>
@@ -968,16 +945,16 @@
         <v>22</v>
       </c>
       <c r="K5" s="6" t="n">
-        <v>220</v>
+        <v>90</v>
       </c>
       <c r="L5" s="6" t="n">
-        <v>380</v>
+        <v>180</v>
       </c>
       <c r="M5" s="4" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="6" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="n">
         <v>2</v>
       </c>
@@ -988,13 +965,13 @@
         <v>1</v>
       </c>
       <c r="D6" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E6" s="4" t="s">
+      <c r="F6" s="4" t="s">
         <v>26</v>
-      </c>
-      <c r="F6" s="4" t="s">
-        <v>27</v>
       </c>
       <c r="G6" s="5" t="s">
         <v>19</v>
@@ -1006,157 +983,157 @@
         <v>21</v>
       </c>
       <c r="J6" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="K6" s="6" t="n">
+        <v>8</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>25</v>
+      </c>
+      <c r="M6" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="K6" s="6" t="n">
+    </row>
+    <row r="7" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="7" t="s">
+        <v>29</v>
+      </c>
+      <c r="C7" s="7" t="n">
+        <v>1</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="F7" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="G7" s="8" t="s">
+        <v>19</v>
+      </c>
+      <c r="H7" s="8" t="s">
+        <v>20</v>
+      </c>
+      <c r="I7" s="8" t="s">
+        <v>21</v>
+      </c>
+      <c r="J7" s="8" t="s">
+        <v>33</v>
+      </c>
+      <c r="K7" s="9" t="n">
         <v>25</v>
       </c>
-      <c r="L6" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="M6" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="C7" s="4" t="n">
+      <c r="L7" s="9" t="n">
+        <v>55</v>
+      </c>
+      <c r="M7" s="7" t="s">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="4" t="s">
+        <v>35</v>
+      </c>
+      <c r="C8" s="4" t="n">
         <v>1</v>
       </c>
-      <c r="D7" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="E7" s="4" t="s">
-        <v>32</v>
-      </c>
-      <c r="F7" s="4" t="s">
-        <v>33</v>
-      </c>
-      <c r="G7" s="5" t="s">
+      <c r="D8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E8" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="F8" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="G8" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="H7" s="5" t="s">
+      <c r="H8" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="I7" s="5" t="s">
+      <c r="I8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J7" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="K7" s="6" t="n">
-        <v>8</v>
-      </c>
-      <c r="L7" s="6" t="n">
-        <v>25</v>
-      </c>
-      <c r="M7" s="4" t="s">
+      <c r="J8" s="4"/>
+      <c r="K8" s="6" t="n">
+        <v>12</v>
+      </c>
+      <c r="L8" s="6" t="n">
         <v>35</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="7" t="s">
-        <v>36</v>
-      </c>
-      <c r="C8" s="7" t="n">
-        <v>1</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>37</v>
-      </c>
-      <c r="E8" s="7" t="s">
+      <c r="M8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="F8" s="7" t="s">
-        <v>39</v>
-      </c>
-      <c r="G8" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="H8" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="J8" s="7"/>
-      <c r="K8" s="9" t="n">
-        <v>12</v>
-      </c>
-      <c r="L8" s="9" t="n">
-        <v>30</v>
-      </c>
-      <c r="M8" s="7" t="s">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="9" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="n">
         <v>5</v>
       </c>
       <c r="B9" s="4" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>1</v>
       </c>
       <c r="D9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="H9" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="I9" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="J9" s="5" t="s">
         <v>42</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="K9" s="6" t="n">
+        <v>15</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>120</v>
+      </c>
+      <c r="M9" s="4" t="s">
         <v>43</v>
       </c>
-      <c r="F9" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="G9" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="J9" s="5" t="s">
-        <v>46</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>40</v>
-      </c>
-      <c r="L9" s="6" t="n">
-        <v>50</v>
-      </c>
-      <c r="M9" s="4" t="s">
-        <v>47</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    </row>
+    <row r="10" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="n">
         <v>6</v>
       </c>
       <c r="B10" s="4" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>49</v>
+        <v>16</v>
       </c>
       <c r="E10" s="4" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="F10" s="4" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="G10" s="5" t="s">
         <v>19</v>
@@ -1167,37 +1144,35 @@
       <c r="I10" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="J10" s="5" t="s">
-        <v>52</v>
-      </c>
+      <c r="J10" s="4"/>
       <c r="K10" s="6" t="n">
-        <v>40</v>
+        <v>0.5</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>120</v>
+        <v>4</v>
       </c>
       <c r="M10" s="4" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="11" customFormat="false" ht="91.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="96" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="7" t="n">
         <v>7</v>
       </c>
       <c r="B11" s="7" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="C11" s="7" t="n">
         <v>1</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="E11" s="7" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="G11" s="8" t="s">
         <v>19</v>
@@ -1210,159 +1185,160 @@
       </c>
       <c r="J11" s="7"/>
       <c r="K11" s="9" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="L11" s="9" t="n">
         <v>20</v>
       </c>
       <c r="M11" s="7" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="J12" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="K12" s="11" t="n">
+        <f aca="false">C5*K5+C6*K6+C8*K8+C9*K9+C10*K10</f>
+        <v>127</v>
+      </c>
+      <c r="L12" s="11" t="n">
+        <f aca="false">C5*L5+C6*L6+C8*L8+C9*L9+C10*L10</f>
+        <v>376</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J13" s="10" t="s">
+        <v>53</v>
+      </c>
+      <c r="K13" s="11" t="n">
+        <f aca="false">C5*K5+C6*K6+C7*K7+C8*K8+C9*K9+C10*K10+C11*K11</f>
+        <v>154</v>
+      </c>
+      <c r="L13" s="11" t="n">
+        <f aca="false">C5*L5+C6*L6+C7*L7+C8*L8+C9*L9+C10*L10+C11*L11</f>
+        <v>451</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="12" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="13" t="s">
+        <v>2</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>55</v>
+      </c>
+      <c r="D16" s="13" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="55.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="14" t="n">
+        <v>1</v>
+      </c>
+      <c r="B17" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="C17" s="14" t="s">
         <v>58</v>
       </c>
-      <c r="K12" s="11" t="n">
-        <f aca="false">SUMPRODUCT(C5:C11,K5:K11)</f>
-        <v>353</v>
-      </c>
-      <c r="L12" s="11" t="n">
-        <f aca="false">SUMPRODUCT(C5:C11,L5:L11)</f>
-        <v>675</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A14" s="12" t="s">
+      <c r="D17" s="14" t="s">
         <v>59</v>
-      </c>
-    </row>
-    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A15" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="B15" s="13" t="s">
-        <v>3</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>60</v>
-      </c>
-      <c r="D15" s="13" t="s">
-        <v>61</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="95.5" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="B16" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="C16" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="D16" s="14" t="s">
-        <v>64</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="14" t="n">
-        <v>2</v>
-      </c>
-      <c r="B17" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="C17" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="D17" s="14" t="s">
-        <v>66</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="14" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="B18" s="14" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
       <c r="C18" s="14" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="D18" s="14" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="14" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B19" s="14" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="C19" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D19" s="14" t="s">
         <v>63</v>
-      </c>
-      <c r="D19" s="14" t="s">
-        <v>70</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="14" t="n">
+        <v>4</v>
+      </c>
+      <c r="B20" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C20" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="D20" s="14" t="s">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="68.65" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="14" t="n">
         <v>5</v>
       </c>
-      <c r="B20" s="14" t="s">
-        <v>71</v>
-      </c>
-      <c r="C20" s="14" t="s">
-        <v>63</v>
-      </c>
-      <c r="D20" s="14" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="14" t="n">
-        <v>6</v>
-      </c>
       <c r="B21" s="14" t="s">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="C21" s="14" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="D21" s="14" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A2:M2"/>
   </mergeCells>
   <hyperlinks>
     <hyperlink ref="G5" r:id="rId1" display="ML · menor preço"/>
     <hyperlink ref="H5" r:id="rId2" display="ML · relevantes"/>
     <hyperlink ref="I5" r:id="rId3" display="Shopee · mais vendidos"/>
-    <hyperlink ref="J5" r:id="rId4" display="Waveshare oficial (US$ 29,99 + frete)"/>
+    <hyperlink ref="J5" r:id="rId4" display="AliExpress — busca ES3C28P"/>
     <hyperlink ref="G6" r:id="rId5" display="ML · menor preço"/>
     <hyperlink ref="H6" r:id="rId6" display="ML · relevantes"/>
     <hyperlink ref="I6" r:id="rId7" display="Shopee · mais vendidos"/>
-    <hyperlink ref="J6" r:id="rId8" display="Busca geral ML (bateria 3,7 V 1000 mAh)"/>
+    <hyperlink ref="J6" r:id="rId8" display="Busca geral ML (alto-falante 8 Ω 2 W)"/>
     <hyperlink ref="G7" r:id="rId9" display="ML · menor preço"/>
     <hyperlink ref="H7" r:id="rId10" display="ML · relevantes"/>
     <hyperlink ref="I7" r:id="rId11" display="Shopee · mais vendidos"/>
-    <hyperlink ref="J7" r:id="rId12" display="Busca geral ML (alto-falante 8 Ω 2 W)"/>
+    <hyperlink ref="J7" r:id="rId12" display="Busca geral ML (bateria 3,7 V 1000 mAh)"/>
     <hyperlink ref="G8" r:id="rId13" display="ML · menor preço"/>
     <hyperlink ref="H8" r:id="rId14" display="ML · relevantes"/>
     <hyperlink ref="I8" r:id="rId15" display="Shopee · mais vendidos"/>
-    <hyperlink ref="J9" r:id="rId16" display="Creative Chance — Neo Deskimon"/>
-    <hyperlink ref="G10" r:id="rId17" display="ML · menor preço"/>
-    <hyperlink ref="H10" r:id="rId18" display="ML · relevantes"/>
-    <hyperlink ref="I10" r:id="rId19" display="Shopee · mais vendidos"/>
-    <hyperlink ref="J10" r:id="rId20" display="Filamento PLA 1,75 mm — busca ML"/>
-    <hyperlink ref="G11" r:id="rId21" display="ML · menor preço"/>
-    <hyperlink ref="H11" r:id="rId22" display="ML · relevantes"/>
-    <hyperlink ref="I11" r:id="rId23" display="Shopee · mais vendidos"/>
+    <hyperlink ref="G9" r:id="rId16" display="ML · menor preço"/>
+    <hyperlink ref="H9" r:id="rId17" display="ML · relevantes"/>
+    <hyperlink ref="I9" r:id="rId18" display="Shopee · mais vendidos"/>
+    <hyperlink ref="J9" r:id="rId19" display="Filamento PLA — busca ML"/>
+    <hyperlink ref="G10" r:id="rId20" display="ML · menor preço"/>
+    <hyperlink ref="H10" r:id="rId21" display="ML · relevantes"/>
+    <hyperlink ref="I10" r:id="rId22" display="Shopee · mais vendidos"/>
+    <hyperlink ref="G11" r:id="rId23" display="ML · menor preço"/>
+    <hyperlink ref="H11" r:id="rId24" display="ML · relevantes"/>
+    <hyperlink ref="I11" r:id="rId25" display="Shopee · mais vendidos"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1388,74 +1364,74 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>75</v>
+        <v>69</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="B2" s="16" t="s">
-        <v>78</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>79</v>
+        <v>73</v>
       </c>
       <c r="B3" s="16" t="s">
-        <v>80</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>74</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>81</v>
+        <v>75</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>82</v>
+        <v>76</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>84</v>
+        <v>78</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>86</v>
+        <v>80</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>88</v>
+        <v>82</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>92</v>
+        <v>86</v>
       </c>
     </row>
   </sheetData>
@@ -1474,7 +1450,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C10"/>
+  <dimension ref="A1:C9"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="40"/>
@@ -1484,122 +1460,110 @@
   <sheetData>
     <row r="1" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="15" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="B1" s="15" t="s">
-        <v>94</v>
+        <v>88</v>
       </c>
       <c r="C1" s="15" t="s">
-        <v>95</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="28.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="16" t="s">
-        <v>96</v>
+        <v>90</v>
       </c>
       <c r="B2" s="17" t="s">
-        <v>97</v>
+        <v>91</v>
       </c>
       <c r="C2" s="16" t="s">
-        <v>98</v>
+        <v>92</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="16" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="B3" s="17" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C3" s="16" t="s">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="B4" s="17" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C4" s="16" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>46</v>
+        <v>99</v>
       </c>
       <c r="B5" s="17" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B6" s="17" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B7" s="17" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B8" s="17" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="C8" s="16" t="s">
-        <v>115</v>
-      </c>
-    </row>
-    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>116</v>
-      </c>
-      <c r="B9" s="17" t="s">
-        <v>117</v>
-      </c>
+        <v>111</v>
+      </c>
+      <c r="B9" s="16"/>
       <c r="C9" s="16" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="10" customFormat="false" ht="41.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="16" t="s">
-        <v>119</v>
-      </c>
-      <c r="B10" s="16"/>
-      <c r="C10" s="16" t="s">
-        <v>120</v>
+        <v>112</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="B2" r:id="rId1" display="https://www.waveshare.com/esp32-s3-touch-amoled-1.75.htm"/>
-    <hyperlink ref="B3" r:id="rId2" display="https://docs.waveshare.com/ESP32-S3-Touch-AMOLED-1.75"/>
-    <hyperlink ref="B4" r:id="rId3" display="https://github.com/waveshareteam/ESP32-S3-Touch-AMOLED-1.75"/>
-    <hyperlink ref="B5" r:id="rId4" display="https://creative-chance.com/en-brl/products/neo-deskimon"/>
-    <hyperlink ref="B6" r:id="rId5" display="https://www.ebay.com/itm/267546467085"/>
-    <hyperlink ref="B7" r:id="rId6" display="https://www.amazon.com/AmpOhm360-Waveshare-Development-Microphones-Interface/dp/B0H97CDMKS"/>
-    <hyperlink ref="B8" r:id="rId7" display="https://lista.mercadolivre.com.br/bateria-3.7v-1000mah"/>
-    <hyperlink ref="B9" r:id="rId8" display="https://lista.mercadolivre.com.br/alto-falante-8-ohms-2w"/>
+    <hyperlink ref="B2" r:id="rId1" display="https://www.lcdwiki.com/2.8inch_ESP32-S3_Display"/>
+    <hyperlink ref="B3" r:id="rId2" display="https://github.com/ngttai/esp32_s3_es3c28p"/>
+    <hyperlink ref="B4" r:id="rId3" display="https://github.com/bmorcelli/Launcher/issues/373"/>
+    <hyperlink ref="B5" r:id="rId4" display="https://github.com/BruceDevices/firmware/pull/2178"/>
+    <hyperlink ref="B6" r:id="rId5" display="https://www.alibaba.com/product-detail/ES3C28P-ES3N28P-2-8-inch-ESP32_1601603512242.html"/>
+    <hyperlink ref="B7" r:id="rId6" display="https://lista.mercadolivre.com.br/bateria-3.7v-1000mah"/>
+    <hyperlink ref="B8" r:id="rId7" display="https://lista.mercadolivre.com.br/alto-falante-8-ohms-2w"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>

</xml_diff>